<commit_message>
qa: FG Golden Path rewritten — A Countertop + B Custom FG (เจดีย์บัว), 32 cases run live 2026-10-06 with screenshots + Excel
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-golden-path-fg.xlsx
+++ b/client-docs/test-cases/emg-o-golden-path-fg.xlsx
@@ -8,10 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="F1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="F2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="F3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="F4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="A1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="A2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="A3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="A4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="B1" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="B2" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="B3" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -459,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C2:D12"/>
+  <dimension ref="C2:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="2" max="2"/>
@@ -470,28 +473,28 @@
     <row r="2">
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>EMG-O — Golden Path: FG Countertop (ชุดที่ 3 จาก 3)</t>
+          <t>EMG-O — Golden Path: FG (A Countertop + B Custom FG เจดีย์บัว)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Empire Stone × Empire Granite — stone_slab_inventory (odoo19-ent-mbx, EE) — post ADR-071/072/073</t>
+          <t>Empire Stone × Empire Granite — stone_slab_inventory (odoo19-ent-mbx, EE) — stone_slab_inventory 2.108.0 + boq_estimation 1.24.0, run live 2026-10-06</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Total test cases: 17</t>
+          <t>Total test cases: 32</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>High / Medium / Low: 15 / 2 / 0</t>
+          <t>High / Medium / Low: 30 / 2 / 0</t>
         </is>
       </c>
     </row>
@@ -510,7 +513,7 @@
     <row r="9">
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>F1 — ใบสั่งขาย Countertop (ท็อปครัว)</t>
+          <t>A1 — ใบสั่งขาย Countertop (ท็อปครัว)</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
@@ -520,7 +523,7 @@
     <row r="10">
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>F2 — ผลิต Countertop (FG Production)</t>
+          <t>A2 — ผลิต Countertop (FG Production)</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
@@ -530,7 +533,7 @@
     <row r="11">
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>F3 — เศษหินกลับเข้าสต็อก</t>
+          <t>A3 — เศษหินกลับเข้าสต็อก</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
@@ -540,10 +543,40 @@
     <row r="12">
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>F4 — ส่งของและเก็บเงิน Countertop</t>
+          <t>A4 — ส่งของ เก็บเงิน และตรวจต้นทุน Countertop</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>B1 — ใบสั่งขาย Custom FG (เจดีย์บัว) พร้อมสูตรจาก BOQ</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>B2 — ตัดหินและประกอบ Custom FG</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>B3 — ส่งของ เก็บเงิน และตรวจต้นทุน Custom FG</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
         <v>4</v>
       </c>
     </row>
@@ -578,7 +611,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F1. ใบสั่งขาย Countertop (ท็อปครัว) — เปิดใบสั่งขาย → ใส่รายการชิ้นงานและงานแปรรูป → ตรวจราคา → Confirm</t>
+          <t>A1. ใบสั่งขาย Countertop (ท็อปครัว) — A</t>
         </is>
       </c>
     </row>
@@ -657,25 +690,25 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>มีลูกค้า (Demo Hotel Customer) และสินค้า Countertop ที่ผูกกับวัสดุแล้ว (GP Block Marble ราคา 12,000 ต่อ m²)</t>
+          <t>มีลูกค้า (A-test-customer) และสินค้า Countertop ที่ผูกกับวัสดุแล้ว (GP Block Marble ราคา 12,000 ต่อ m²)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
           <t>1. เปิดแอป Sales &gt; Orders &gt; Quotations &gt; New
 2. เลือก Customer
-3. กด "Add a product" เลือกสินค้า Countertop
+3. กด "Add a product" เลือกสินค้า Countertop (GP Block Marble)
 4. กด Save</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>Customer = Demo Hotel Customer · Product = GP Block Marble</t>
+          <t>Customer = A-test-customer · Product = GP Block Marble</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบเสนอราคาใหม่ (ตัวอย่างจริง S00178) มีบรรทัดสินค้า GP Block Marble หน่วย m² ราคา 12,000.00 ต่อหน่วย และมีไอคอนรายการชิ้นงานบนบรรทัด</t>
+          <t>ใบเสนอราคาใหม่ (ตัวอย่างจริง S00193) มีบรรทัดสินค้า GP Block Marble หน่วย m² ราคา 12,000.00 ต่อหน่วย และมีไอคอนรายการชิ้นงานบนบรรทัด</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -712,8 +745,8 @@
       <c r="D5" s="7" t="inlineStr">
         <is>
           <t>1. กดไอคอนรายชิ้น (ไอคอนรายการ) บนบรรทัดสินค้า
-2. กดปุ่ม "New" แล้วกรอกรหัสชิ้น กว้าง ยาว และจำนวน
-3. ทำซ้ำจนครบทุกชิ้น แล้วปิดหน้าต่าง</t>
+2. กดปุ่ม "New" แล้วกรอกรหัสชิ้น กว้าง ยาว และจำนวน แล้วกด Save
+3. ทำซ้ำจนครบทุกชิ้น</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -900,7 +933,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F2. ผลิต Countertop (FG Production) — เปิดใบสั่งผลิต → ระบบเลือก Slab ให้ → ย้ายไปสถานีผลิต → Confirm → บันทึกชิ้นที่ตัดได้ + เศษ → Complete</t>
+          <t>A2. ผลิต Countertop (FG Production) — A</t>
         </is>
       </c>
     </row>
@@ -995,7 +1028,7 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบสั่งผลิต EG01/STFG/00034 (Draft) — พื้นที่งาน 3.48 ตร.ม. · ต้องใช้รวมเผื่อเสีย 3.83 ตร.ม. (เผื่อเสีย 10% ตามที่ตั้งไว้ในบริษัท) · ระบบเลือก Slab ให้เอง 2 แผ่น (BLK-26-0006-3 และ -4 แผ่นละ 3.75 ตร.ม.) รวม 7.50 ตร.ม. พอสำหรับงาน</t>
+          <t>ใบสั่งผลิต EG01/STFG/00046 (Draft) — พื้นที่งาน 3.48 ตร.ม. · ต้องใช้รวมเผื่อเสีย 3.83 ตร.ม. (เผื่อเสีย 10%) · ระบบเลือก Slab ให้เอง 2 แผ่น (BLK-26-0006-9 และ -10 แผ่นละ 3.75 ตร.ม.) รวม 7.50 ตร.ม. พอสำหรับงาน · มีกล่องข้อความอธิบายว่าจำนวนในแท็บ Components ตอนนี้เป็นค่าตั้งต้นจากสูตร จะตรงกับ Slab ที่เลือกหลัง Confirm</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1003,11 +1036,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>แถบเตือนสีส้มและแท็บ Components ยังแสดงแผ่นมาตรฐานตามสูตร (Honed 3 cm, Not Available) ไว้ก่อน — จะถูกแทนที่ด้วยแผ่นที่เลือกจริงตอน Confirm เป็นแค่ข้อความ ไม่กระทบการทำงาน</t>
-        </is>
-      </c>
+      <c r="H4" s="7" t="n"/>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
@@ -1083,7 +1112,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ใบสั่งผลิตเป็น Confirmed · ข้อความนำทางสีฟ้าบอกขั้นถัดไป (กรอก FG Output แล้วกด Complete FG Production)</t>
+          <t>ใบสั่งผลิตเป็น Confirmed · ข้อความนำทางสีฟ้าบอกขั้นถัดไป (กรอก FG Output แล้วกด Complete FG Production) · จำนวนแผ่นในแท็บ Components ตรงกับ Slab ที่เลือกจริง</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1093,7 +1122,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>แท็บ Work Orders มี 4 ขั้นตอน (ตัดตามแบบ → ทำขอบ → เจาะ/ตัดช่อง → ตรวจก่อนส่ง) แต่ไม่ต้องกด Start ทีละขั้นก็ปิดงานได้ ในชุดนี้ข้ามส่วนจับเวลา — ขั้นตอนเหล่านี้ไม่ได้ทดสอบ · ช่อง Component Status ยังขึ้น Not Available แม้ย้าย Slab มาแล้ว แต่ไม่ขวางการ Complete</t>
+          <t>แท็บ Work Orders มี 4 ขั้นตอน (ตัดตามแบบ → ทำขอบ → เจาะ/ตัดช่อง → ตรวจก่อนส่ง) แต่ไม่ต้องกด Start ทีละขั้นก็ปิดงานได้ ในชุดนี้ข้ามส่วนจับเวลา — ขั้นตอนเหล่านี้ไม่ได้ทดสอบ · ต้อง Confirm ก่อนจึงกด Complete ได้ (ถ้ายังเป็น Draft ระบบจะไม่ให้ปิดงาน)</t>
         </is>
       </c>
       <c r="I6" s="7" t="n"/>
@@ -1173,7 +1202,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>เศษจาก -3: 1.20 × 1.20 (1 ชิ้น) · เศษจาก -4: 2.00 × 1.25 (1 ชิ้น)</t>
+          <t>เศษจาก -10: 1.20 × 1.20 (1 ชิ้น) · เศษจาก -9: 2.00 × 1.25 (1 ชิ้น)</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -1220,7 +1249,7 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>แจ้งเตือนสีเขียว "Complete FG Production สำเร็จ EG01/STFG/00034 ผลิตสำเร็จ 3.48 หน่วย" · ใบสั่งผลิตขึ้น Done · Quantity 3.48 / 3.48 · Slab 2 แผ่นถูกใช้ไป (Consumed 2.00) · ได้ FG 3 Lot ตามขนาดชิ้น (FG-EG01/STFG/00034-01 ถึง -03) เข้าสต็อกคลัง และต้นทุนรวม 1,153.44 บาท (331.45 ต่อ m²) = ค่า Slab 2,430.00 หักส่วนของเศษ 1,276.56</t>
+          <t>แจ้งเตือนสีเขียว "Complete FG Production สำเร็จ EG01/STFG/00046 ผลิตสำเร็จ 3.48 หน่วย" · ใบสั่งผลิตขึ้น Done · ได้ FG 3 Lot ตามขนาดชิ้น (FG-EG01/STFG/00046-01 ถึง -03) เข้าโซน EG01/Stock/Stone FG และต้นทุนวัสดุ 1,153.44 บาท (331.45 ต่อ m²) = ค่า Slab 2,430.00 หักส่วนของเศษ 1,276.56 · เศษได้ Lot ของตัวเอง (OC-EG01/STFG/00046-01 ต้นทุน 466.56, -02 ต้นทุน 810.00)</t>
         </is>
       </c>
       <c r="G9" s="7" t="inlineStr">
@@ -1228,11 +1257,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
-        <is>
-          <t>หลังปิดงาน แท็บ Components ยังมีแถวแผ่นมาตรฐานตามสูตร (Honed 3 cm) ที่ Consumed 0.00 คู่กับแถวแผ่นจริงที่ใช้ (Polished 2 cm, Consumed 2.00) — เป็นแค่การแสดงผล ไม่กระทบสต็อก</t>
-        </is>
-      </c>
+      <c r="H9" s="7" t="n"/>
       <c r="I9" s="7" t="n"/>
       <c r="J9" s="7" t="n"/>
       <c r="K9" s="7" t="n"/>
@@ -1272,7 +1297,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F3. เศษหินกลับเข้าสต็อก — เศษที่เหลือกลายเป็น Lot ใหม่รอตรวจ → ตรวจแล้วนำกลับไปขาย</t>
+          <t>A3. เศษหินกลับเข้าสต็อก — A</t>
         </is>
       </c>
     </row>
@@ -1356,19 +1381,18 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิดแอป Stone Slab &gt; Slabs &gt; All Slabs
-2. ลบตัวกรอง "Available" ออก แล้วค้นหา "OC-EG01/STFG/00034"
-3. เปิดเศษ OC-EG01/STFG/00034-01 ดู Location, Status และต้นทุน</t>
+          <t>1. เปิดแอป Stone Slab &gt; Slabs &gt; Slabs Pending Inspection
+2. ค้นหา "OC-EG01/STFG/00046" แล้วเปิดเศษก้อนแรก ดู Location, Status และต้นทุน</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>OC-EG01/STFG/00034-01</t>
+          <t>OC-EG01/STFG/00046-01</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>เศษแต่ละก้อนเป็น Lot ของตัวเอง ขนาดจริง (1.20 × 1.20 × 0.02 ม. = 1.44 ตร.ม.) · อยู่ที่ Stone Inventory/Returned - Inspect · Status "Returned - Pending Inspection" · ต้นทุน 466.56 บาท (ส่วนแบ่งตามพื้นที่) — ก้อนที่ 2 (2.00 × 1.25) ต้นทุน 810.00 บาท</t>
+          <t>เศษแต่ละก้อนเป็น Lot ของตัวเอง ขนาดจริง (1.20 × 1.20 × 0.02 ม. = 1.44 ตร.ม.) · Status "Returned - Pending Inspection" · ต้นทุน 466.56 บาท (ส่วนแบ่งตามพื้นที่) — ก้อนที่ 2 (2.00 × 1.25) ต้นทุน 810.00 บาท</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1407,12 +1431,12 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>OC-EG01/STFG/00034-01 และ -02</t>
+          <t>OC-EG01/STFG/00046-01 และ -02</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>สถานะเปลี่ยนเป็น Available · Location เป็น Stone Inventory/Stone Available · ปุ่มตรวจแล้ว/ชำรุดหายไป · ต้นทุนยังเป็น 466.56 และ 810.00 บาทเท่าเดิม — เศษกลับมาขายเป็น Slab ขนาดเล็กได้</t>
+          <t>สถานะเปลี่ยนเป็น Available · กลับไปอยู่ Stone Available · ปุ่มตรวจแล้ว/ชำรุดหายไป · ต้นทุนยังเป็น 466.56 และ 810.00 บาทเท่าเดิม — เศษกลับมาขายเป็น Slab ขนาดเล็กได้</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1439,6 +1463,324 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>A4. ส่งของ เก็บเงิน และตรวจต้นทุน Countertop — A</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>ข้อมูลตัวอย่าง (Sample Data)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Status (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Tester</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-14</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>เปิดใบส่งของ ตรวจว่าระบบจอง FG ถูก Lot</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-11 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิด Sales Order กดสมาร์ทปุ่ม "Delivery"
+2. กดปุ่ม Check Availability (ถ้ายังไม่จอง)
+3. ที่แถวสินค้า กด "Details" ดูรายการ Lot</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>ใบส่งของ EG01/OUT/00076 · Detailed Operations ระบุ Lot ครบ 3 แถวจากโซน EG01/Stock/Stone FG: FG-EG01/STFG/00046-01 (1.56 m²), -02 (0.72 m²), -03 (1.20 m²) รวม 3.48 m² ตรงกับที่สั่ง — ไม่ต้องสแกนหรือเลือก Lot เอง</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="n"/>
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="n"/>
+      <c r="L4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-15</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>กด Validate ส่งของ</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-14 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม Validate บนใบส่งของ</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>ใบส่งของขึ้น Done · Quantity 3.48 จาก Demand 3.48 · มี Effective Date · ปุ่ม Traceability ปรากฏ (ย้อนดูได้ว่าสินค้ามาจาก Slab แผ่นไหน)</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-16</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>สร้างใบแจ้งหนี้จาก Sales Order</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-15 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>1. กลับไปที่ Sales Order กดปุ่ม "Create Invoice"
+2. เลือก "Regular invoice" แล้วกด "Create Draft"</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Regular invoice</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>ได้ใบแจ้งหนี้ฉบับร่าง 4 บรรทัดตรงกับ Sales Order: GP Block Marble 3.48 m² = 41,760.00 · งานขอบ 3.60 ม. = 1,260.00 · งานเจาะช่องเตา 1,500.00 · งานเจาะช่องซิงค์ 1,200.00 — รวม 45,720.00 + VAT 3,200.40 = 48,920.40 บาท</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-17</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>กด Confirm ใบแจ้งหนี้ให้ Posted</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-16 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม Confirm บนใบแจ้งหนี้</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>ใบแจ้งหนี้ INV/2026/00011 เป็น Posted · ยอดค้างชำระ 48,920.40 บาท · บัญชีบันทึกรายได้ 45,720.00 + VAT 3,200.40 และต้นทุนขาย (COGS) 1,153.44 เท่ากับต้นทุน FG ที่ตัดออกจากคลัง · บรรทัดหินติดแท็ก Analytic ทำให้รายงานอ้างอิงกลับไปถึง Block ต้นทางได้</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-18</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>ตรวจต้นทุนรวมของ FG ไม่ต่ำกว่า 50% ของยอดขายหิน</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-11 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดแอป Accounting &gt; Journal Entries ค้นหา "FG Production Labor — EG01/STFG/00046"
+2. ดูบัญชีเดบิต/เครดิตและยอดเงิน</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>รายการบัญชี MISC/2026/10/0003: เดบิต 511120 COGS - FG Production (Fabrication) 19,378.56 / เครดิต 212300 Accrued Expenses 19,378.56 (ค่าวัสดุสิ้นเปลือง 348.00 ลงอีกรายการแยก) · ต้นทุนรวม = วัสดุ 1,153.44 + วัสดุสิ้นเปลือง 348.00 + ค่าแรง 19,378.56 = 20,880.00 = 50% ของยอดขายหิน 41,760.00 พอดี</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>ค่าแรงและค่าแปรรูปเป็นอัตรามาตรฐานชั่วคราว (หมวด Countertop ม² ละ 1,500 + วัสดุสิ้นเปลือง 100) ถ้าต้นทุนรวมยังไม่ถึง 50% ของยอดขาย ระบบเติมส่วนต่างเป็นค่าแรง/แปรรูปให้ — ปรับสัดส่วนได้ที่ค่าระบบ stone_slab_inventory.fg_min_cost_ratio · ค่าแรงลงบัญชีตอนผลิตเสร็จ ต้นทุนวัสดุลงตอนส่งของ/ออกใบแจ้งหนี้</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1464,7 +1806,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>F4. ส่งของและเก็บเงิน Countertop — ใบส่งของ → Validate → ใบแจ้งหนี้ → Post</t>
+          <t>B1. ใบสั่งขาย Custom FG (เจดีย์บัว) พร้อมสูตรจาก BOQ — B</t>
         </is>
       </c>
     </row>
@@ -1533,33 +1875,35 @@
     <row r="4" ht="60" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>TC-GP-FG-14</t>
+          <t>TC-GP-FG-19</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>เปิดใบส่งของ ตรวจว่าระบบจอง FG ถูก Lot</t>
+          <t>สร้างใบสั่งขาย แล้วเลือกสินค้า Custom FG จำนวนเป็นชิ้น</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-GP-FG-11 เสร็จแล้ว</t>
+          <t>มีลูกค้า (A-test-customer) และสินค้า เจดีย์บัว (Custom FG) · มี BOQ ที่เตรียมสูตรไว้แล้ว (BOQ0023: หิน NERO + GP Block Marble พร้อมรายชิ้น, กาว, ซีลแลนท์)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>1. เปิด Sales Order กดสมาร์ทปุ่ม "Delivery"
-2. ที่แถวสินค้า กด "Details" ดูรายการ Lot</t>
+          <t>1. เปิดแอป Sales &gt; Orders &gt; Quotations &gt; New
+2. เลือก Customer
+3. กด "Add a product" เลือก เจดีย์บัว ใส่จำนวน 3
+4. กด Save</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Customer = A-test-customer · Product = เจดีย์บัว · Quantity = 3</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของ EG01/OUT/00062 สถานะ Ready · Product Availability = Available · Detailed Operations ระบุ Lot ครบ 3 แถว: FG-EG01/STFG/00034-01 (1.56 m²), -02 (0.72 m²), -03 (1.20 m²) รวม 3.48 m² ตรงกับที่สั่ง — ไม่ต้องสแกนหรือเลือก Lot เอง</t>
+          <t>ใบเสนอราคา S00194 มีบรรทัดเจดีย์บัว 3 ชิ้น × 50,000.00 = 150,000.00 ก่อน VAT · มีไอคอน "โหลด BOQ" และ "ดูสูตร" บนบรรทัด</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
@@ -1567,7 +1911,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H4" s="7" t="n"/>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>สินค้า Custom FG (ติ๊ก "เป็น Custom FG" ที่สินค้า) ไม่ผูกกับวัสดุเดียว ราคาตั้งไว้ที่สินค้า (เจดีย์บัว 50,000 ต่อชิ้น) จำนวนในบรรทัดคือ "จำนวนชิ้นสำเร็จรูป" และ Sales แก้ราคาได้</t>
+        </is>
+      </c>
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="7" t="n"/>
       <c r="K4" s="7" t="n"/>
@@ -1576,32 +1924,34 @@
     <row r="5" ht="60" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>TC-GP-FG-15</t>
+          <t>TC-GP-FG-20</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>กด Validate ส่งของ</t>
+          <t>โหลด BOQ เป็นสูตรของบรรทัดนี้</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-GP-FG-14 เสร็จแล้ว</t>
+          <t>ทำ TC-GP-FG-19 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม Validate บนใบส่งของ</t>
+          <t>1. กดไอคอน "โหลด BOQ" บนบรรทัดเจดีย์บัว
+2. เลือก BOQ ที่เตรียมไว้ (BOQ0023)
+3. กดปุ่ม "โหลด BOQ"</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>BOQ = BOQ0023</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>ใบส่งของขึ้น Done · Quantity 3.48 จาก Demand 3.48 · มี Effective Date · ปุ่ม Traceability ปรากฏ (ย้อนดูได้ว่าสินค้ามาจาก Slab แผ่นไหน)</t>
+          <t>ระบบคัดลอกบรรทัดหิน (พร้อมรายชิ้น) และวัสดุสิ้นเปลือง จาก BOQ เข้ามาเป็นสูตรของบรรทัดนี้ (ปริมาณต่อชิ้นงาน 1 หน่วย) — แก้ BOQ ภายหลังไม่กระทบสูตรที่โหลดแล้ว · บรรทัดใบสั่งขายแสดงคอลัมน์ ต้นทุน/ชิ้น (ประมาณ) และ Margin/ชิ้น (ประมาณ)</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
@@ -1618,33 +1968,316 @@
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>TC-GP-FG-16</t>
+          <t>TC-GP-FG-21</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>สร้างใบแจ้งหนี้จาก Sales Order</t>
+          <t>ตรวจสูตรและต้นทุนประมาณต่อชิ้น</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-GP-FG-15 เสร็จแล้ว</t>
+          <t>ทำ TC-GP-FG-20 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>1. กลับไปที่ Sales Order กดปุ่ม "Create Invoice"
-2. เลือก "Regular invoice" แล้วกด "Create Draft"</t>
+          <t>1. กดไอคอน "ดูสูตร / ต้นทุน" บนบรรทัด</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Regular invoice</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>ได้ใบแจ้งหนี้ฉบับร่าง 4 บรรทัดตรงกับ Sales Order: GP Block Marble 3.48 m² = 41,760.00 · งานขอบ 3.60 ม. = 1,260.00 · งานเจาะช่องเตา 1,500.00 · งานเจาะช่องซิงค์ 1,200.00 — รวม 45,720.00 + VAT 3,200.40 = 48,920.40 บาท</t>
+          <t>ตารางสูตร 4 แถว: NERO RUSTENBURG 0.36 ม² (เผื่อเสีย 10%) = 637.96 · GP Block Marble 0.54 ม² (เผื่อเสีย 10%) = 192.46 · กาว/epoxy 0.90 ม² = 108.00 · ซีลแลนท์ 0.90 ม² = 22.50 · รวมต้นทุนประมาณ 960.92 บาทต่อชิ้น · รายชิ้นของแต่ละหิน (GP-01, GP-02, GP-03) แสดงในคอลัมน์ขวา</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>ต้นทุนในหน้านี้เป็น "ประมาณ" คำนวณจากราคา Rate ใน BOQ × ปริมาณ (รวมเผื่อเสีย) ไม่ใช่ต้นทุนจริงของ Slab — ต้นทุนจริงจะเห็นที่ Serial หลังผลิต (TC-GP-FG-30)</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-22</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>กด Confirm — ระบบสร้างใบสั่งผลิตให้ครบ</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-21 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม Confirm
+2. กดสมาร์ทปุ่ม "FG Production" ดูใบสั่งผลิตที่ระบบสร้าง</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>ใบเสนอราคาเป็น Sales Order · ระบบสร้างใบสั่งผลิตฉบับร่าง 3 ใบ: งานประกอบ EG01/STFG/00047 (เจดีย์บัว 3 ชิ้น) + ใบตัดหิน NERO EG01/STCPL/00011 (6 ชิ้น) + ใบตัดหิน GP Block Marble EG01/STCPL/00012 (3 ชิ้น) — จำนวนชิ้นตัด = ชิ้นต่อ 1 หน่วย × 3 หน่วย (เช่น "GP-01 #2")</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Confirm ผ่านเสมอแม้หินในสต็อกไม่พอ (ใบสั่งผลิตจะค้างเป็นฉบับร่างพร้อมเตือน) · ถ้าบรรทัด Custom FG ไม่มีสูตร ระบบไม่ให้ Confirm</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>B2. ตัดหินและประกอบ Custom FG — B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>ข้อมูลตัวอย่าง (Sample Data)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Status (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Tester</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-23</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>เปิดใบตัดหินของหินชนิดแรก (NERO RUSTENBURG)</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-22 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดแอป Manufacturing เปิดใบตัดหิน EG01/STCPL/00011 (หรือจากสมาร์ทปุ่มบน Assembly)</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>ใบตัดหิน Draft · ผลผลิต "เทาดำอัฟริกา/NERO RUSTENBURG - Cutting Plan WIP" 6 ชิ้น · ผูกกับงานประกอบ EG01/STFG/00047 (For Assembly) · มีข้อความนำทางให้กด "ย้ายด่วน" ก่อน Confirm</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>ตอนยังเป็น Draft แท็บ Components แสดงจำนวน 6 ตามสูตร แต่หลัง Confirm ระบบใช้ Slab จริง 1 แผ่นต่อชนิดหิน (มีกล่องข้อความอธิบายบนหน้า) · ต้อง Confirm ก่อนจึงกด Complete ได้</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="n"/>
+      <c r="L4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-24</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>ย้ายหินเข้าไลน์ผลิตและ Confirm ใบตัดหิน</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-23 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม "ย้ายด่วน (Move to Production)" (ถ้าหินยังอยู่ที่ Stone Available)
+2. กดปุ่ม Confirm</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>ใบตัดหินเป็น Confirmed · แท็บ Components แสดงแผ่น NERO ที่ใช้ 1.00 แผ่น (Available) · ข้อความนำทางบอกให้กรอกขนาดจริงในแท็บ Planned/Actual Pieces แล้วกด Complete Cutting Plan</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-25</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>กรอกขนาดชิ้นที่ตัดได้จริงและกด Complete Cutting Plan (NERO)</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-24 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดแท็บ "Planned/Actual Pieces"
+2. กรอก Actual L / H / Thickness ของทุกชิ้น
+3. กดปุ่ม "Complete Cutting Plan"</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>ตัดได้ตรงแบบ: 0.30 × 0.60 ม. หนา 0.02 ม. ทั้ง 6 ชิ้น</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>ใบตัดหินขึ้น Done · ได้ WIP Lot CUT-EG01/STCPL/00011 รวม 6 ชิ้น มูลค่า 2,899.80 บาท (ต้นทุน Slab แผ่นที่ใช้) อยู่ที่ Stone Production</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
@@ -1661,32 +2294,398 @@
     <row r="7" ht="60" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>TC-GP-FG-17</t>
+          <t>TC-GP-FG-26</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>กด Confirm ใบแจ้งหนี้ให้ Posted</t>
+          <t>ตัดหินชนิดที่สอง (GP Block Marble) ให้เสร็จเช่นเดียวกัน</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>ทำ TC-GP-FG-16 เสร็จแล้ว</t>
+          <t>ทำ TC-GP-FG-25 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม Confirm บนใบแจ้งหนี้</t>
+          <t>1. เปิดใบตัดหิน EG01/STCPL/00012
+2. ทำเหมือนข้างต้น: Confirm → กรอกขนาดจริง → Complete Cutting Plan</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
+          <t>ตัดได้ตรงแบบ: 0.60 × 0.90 ม. หนา 0.02 ม. 3 ชิ้น</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>ใบตัดหินขึ้น Done · ได้ WIP Lot CUT-EG01/STCPL/00012 รวม 3 ชิ้น มูลค่า 1,215.00 บาท (ต้นทุน Slab 1 แผ่น)</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-27</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Confirm งานประกอบ — ระบบดึง WIP และวัสดุสิ้นเปลือง</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-26 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดงานประกอบ EG01/STFG/00047
+2. กดปุ่ม Confirm</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>งานประกอบเป็น Confirmed · ช่อง Cutting Plan Lots (Stage 2) แสดง CUT-EG01/STCPL/00011 และ 00012 · แท็บ Components: WIP NERO 6, WIP GP 3, กาว 2.70 ม², ซีลแลนท์ 2.70 ม² (0.90 × 3 ชิ้น) พร้อมใช้</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>งานประกอบ Confirm ไม่ได้จนกว่าใบตัดหินที่ผูกกันทุกใบจะ Done · กาวและซีลแลนท์ต้องมีสต็อกที่ Stone Production (ในชุดทดสอบรับเข้าไว้ 100 หน่วยต่อรายการ) ถ้าไม่มีสต็อก ต้นทุนวัสดุส่วนนี้จะไม่เข้า Serial</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="n"/>
+      <c r="J8" s="7" t="n"/>
+      <c r="K8" s="7" t="n"/>
+      <c r="L8" s="7" t="n"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-28</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>กด Produce All — ได้ Serial 1 ตัวต่อชิ้น</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-27 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม "Produce All" บนงานประกอบ</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>งานประกอบขึ้น Done · Quantity 3.00 / 3.00 · ได้ Serial Numbers 3 ตัว (CB-00013, CB-00014, CB-00015) อยู่ที่ EG01/Stock/Stone FG · วัสดุทุกรายการถูกใช้ครบ (Consumed 6 / 3 / 2.70 / 2.70) · ต้นทุนแต่ละ Serial 1,502.10 บาท (= WIP 4,114.80 + วัสดุสิ้นเปลือง 391.50 หาร 3) · ปุ่ม Serial Numbers / Traceability ย้อนดูได้ถึง Slab ต้นทาง</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+      <c r="J9" s="7" t="n"/>
+      <c r="K9" s="7" t="n"/>
+      <c r="L9" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>B3. ส่งของ เก็บเงิน และตรวจต้นทุน Custom FG — B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>TC ID</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>Precondition</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>ข้อมูลตัวอย่าง (Sample Data)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="I3" s="6" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>Status (Pass/Fail)</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Tester</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-29</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>เปิดใบส่งของ ตรวจว่าระบบจอง Serial ของงานนี้ให้เอง</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-28 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิด Sales Order S00194 กดสมาร์ทปุ่ม "Delivery"
+2. ที่แถวสินค้า กด "Details" ดูรายการ Serial</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>ใบส่งของ EG01/OUT/00077 พร้อมส่ง (Ready) · Detailed Operations ระบุ Serial ครบ 3 แถวจากโซน EG01/Stock/Stone FG: CB-00013, CB-00014, CB-00015 (ชิ้นละ 1) — ไม่ต้องสแกนหรือเลือกเอง</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>Serial ที่ผลิตให้ใบขายใบไหนจะถูกผูกกับใบส่งของของใบขายนั้น — ใบส่งของของใบขายอื่นที่ค้างอยู่จะไม่หยิบไป</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="n"/>
+      <c r="J4" s="7" t="n"/>
+      <c r="K4" s="7" t="n"/>
+      <c r="L4" s="7" t="n"/>
+    </row>
+    <row r="5" ht="60" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-30</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>กด Validate ส่งของ</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-29 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม Validate บนใบส่งของ</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>ใบส่งของขึ้น Done · Quantity 3.00 จาก Demand 3.00 · Serial ทั้ง 3 ตัวออกจากโซน Stone FG ไปที่ลูกค้า</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+      <c r="J5" s="7" t="n"/>
+      <c r="K5" s="7" t="n"/>
+      <c r="L5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-31</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>ออกใบแจ้งหนี้และ Post</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-30 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>1. กลับไปที่ Sales Order กดปุ่ม "Create Invoice"
+2. เลือก "Regular invoice" แล้วกด "Create Draft"
+3. กดปุ่ม Confirm บนใบแจ้งหนี้</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>Regular invoice</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>ใบแจ้งหนี้ INV/2026/00012 เป็น Posted · เจดีย์บัว 3 ชิ้น × 50,000.00 = 150,000.00 + VAT 10,500.00 = 160,500.00 บาท · บัญชีบันทึกรายได้ 150,000.00 และต้นทุนขาย 4,506.30 = ต้นทุน Serial 3 ตัวที่ตัดออกจากคลัง FG</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n"/>
+      <c r="I6" s="7" t="n"/>
+      <c r="J6" s="7" t="n"/>
+      <c r="K6" s="7" t="n"/>
+      <c r="L6" s="7" t="n"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>TC-GP-FG-32</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>ตรวจต้นทุนรวมของ Custom FG ไม่ต่ำกว่า 50% ของยอดขาย</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>ทำ TC-GP-FG-28 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>1. เปิดแอป Accounting &gt; Journal Entries ค้นหา "FG Production Labor — EG01/STFG/00047"
+2. ดูบัญชีเดบิต/เครดิตและยอดเงิน</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>ใบแจ้งหนี้ INV/2026/00006 เป็น Posted · ยอดค้างชำระ 48,920.40 บาท · บรรทัดหินติดแท็ก Analytic (Sale / Marble / GP Block Marble / BLK-26-0006) ทำให้รายงานต้นทุนอ้างอิงกลับไปถึง Block ต้นทางได้ · มีปุ่ม Pay และ Credit Note พร้อมใช้</t>
+          <t>รายการบัญชี MISC/2026/10/0005: เดบิต 511120 COGS - FG Production (Fabrication) 70,493.70 / เครดิต 212300 Accrued Expenses 70,493.70 · ต้นทุนรวม = วัสดุ+วัสดุสิ้นเปลือง 4,506.30 + ค่าแรง 70,493.70 = 75,000.00 = 50% ของยอดขาย 150,000.00 พอดี</t>
         </is>
       </c>
       <c r="G7" s="7" t="inlineStr">
@@ -1694,7 +2693,11 @@
           <t>High</t>
         </is>
       </c>
-      <c r="H7" s="7" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>ค่าแรงงานแกะสลัก/ประกอบเป็นอัตรามาตรฐานชั่วคราว (หมวด Custom ชิ้นละ 10,000) ระบบเติมส่วนต่างให้ต้นทุนรวมถึง 50% ของยอดขาย — เป็นตัวเลขตั้งต้นเพื่อใช้ทดสอบ ต้องปรับเป็นค่าแรงจริงของโรงงานก่อนใช้งานจริง · งานแปรรูปแบบบริการ (บรรทัดบริการในใบขาย) ยังไม่มีต้นทุนของตัวเอง</t>
+        </is>
+      </c>
       <c r="I7" s="7" t="n"/>
       <c r="J7" s="7" t="n"/>
       <c r="K7" s="7" t="n"/>

</xml_diff>